<commit_message>
auto: scan 2026-10-03 12:08 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1045,6 +1045,63 @@
       <c r="O9" s="3" t="inlineStr">
         <is>
           <t>2026-07-22 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5229022</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 100°F or higher on October 5?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.4149</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.1249</v>
+      </c>
+      <c r="H10" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="J10" t="n">
+        <v>75</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-10-03 15:08</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:00</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1436,6 +1493,36 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5229022</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.4149</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.1249</v>
+      </c>
+      <c r="E10" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1447,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1691,6 +1778,31 @@
         <v>0.1077</v>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5229022</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 100°F or high</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1249</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
@@ -1734,7 +1846,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1918,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3884</t>
+          <t>0.3591</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2144,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2446,6 +2558,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5229022</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 100°F or high</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>65</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-10-05 15:23 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -1049,57 +1049,63 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>5229022</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 100°F or higher on October 5?</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="3" t="n">
         <v>0.4149</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="3" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="3" t="n">
         <v>0.1249</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="3" t="n">
         <v>53.1</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="3" t="n">
         <v>0.292</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>181.85</v>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>2026-10-03 15:08</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>2026-10-05 15:00</t>
         </is>
@@ -1513,10 +1519,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>181.85</v>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-10-05 15:00</t>
@@ -1858,7 +1866,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1878,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1902,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>44.4%</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1914,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$406.66</t>
+          <t>$588.50</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2103,6 +2111,23 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>588.5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10588.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2156,7 +2181,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2193,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>44.4%</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2205,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$406.66</t>
+          <t>$588.50</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2217,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$50.83</t>
+          <t>$65.39</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2229,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$318.29</t>
+          <t>$302.90</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2241,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.160</t>
+          <t>0.216</t>
         </is>
       </c>
     </row>

</xml_diff>